<commit_message>
Sprint 2.6 - Poster optisch verbessern
</commit_message>
<xml_diff>
--- a/Excel/Terminefussball_2026_Frühjahr.xlsx
+++ b/Excel/Terminefussball_2026_Frühjahr.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTB\asv-neufeld\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTB\ASV-Manager\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC7DA4B-1AB1-4638-9D58-F1BB6873CBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9189919-EA7B-4EFC-B69E-6D3BA7221292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="941" uniqueCount="246">
   <si>
     <t>Mannschaft</t>
   </si>
@@ -777,6 +777,12 @@
   </si>
   <si>
     <t>abgesagt</t>
+  </si>
+  <si>
+    <t>ART</t>
+  </si>
+  <si>
+    <t>Spiel</t>
   </si>
 </sst>
 </file>
@@ -4171,7 +4177,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E571BD24-40DC-4066-8BBA-CF3C23365042}">
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="108"/>
@@ -4184,7 +4190,7 @@
     <col min="10" max="10" width="11.5546875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="108" t="s">
         <v>132</v>
       </c>
@@ -4218,8 +4224,11 @@
       <c r="K1" s="108" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" s="108" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B2" s="105">
         <f>'Nach Mannschaften sortiert'!D2</f>
         <v>46096</v>
@@ -4257,8 +4266,11 @@
       <c r="K2" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B3" s="105">
         <f>'Nach Mannschaften sortiert'!D3</f>
         <v>46102</v>
@@ -4296,8 +4308,11 @@
       <c r="K3" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L3" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B4" s="105">
         <f>'Nach Mannschaften sortiert'!D4</f>
         <v>46109</v>
@@ -4335,8 +4350,11 @@
       <c r="K4" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L4" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B5" s="105">
         <f>'Nach Mannschaften sortiert'!D5</f>
         <v>46116</v>
@@ -4374,8 +4392,11 @@
       <c r="K5" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L5" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B6" s="105">
         <f>'Nach Mannschaften sortiert'!D6</f>
         <v>46124</v>
@@ -4413,8 +4434,11 @@
       <c r="K6" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L6" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B7" s="105">
         <f>'Nach Mannschaften sortiert'!D7</f>
         <v>46130</v>
@@ -4452,8 +4476,11 @@
       <c r="K7" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L7" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B8" s="105">
         <f>'Nach Mannschaften sortiert'!D8</f>
         <v>46136</v>
@@ -4491,8 +4518,11 @@
       <c r="K8" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L8" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B9" s="105">
         <f>'Nach Mannschaften sortiert'!D9</f>
         <v>46144</v>
@@ -4530,8 +4560,11 @@
       <c r="K9" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L9" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="105">
         <f>'Nach Mannschaften sortiert'!D10</f>
         <v>46151</v>
@@ -4569,8 +4602,11 @@
       <c r="K10" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L10" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B11" s="105">
         <f>'Nach Mannschaften sortiert'!D11</f>
         <v>46157</v>
@@ -4608,8 +4644,11 @@
       <c r="K11" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L11" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B12" s="105">
         <f>'Nach Mannschaften sortiert'!D12</f>
         <v>46166</v>
@@ -4647,8 +4686,11 @@
       <c r="K12" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L12" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B13" s="105">
         <f>'Nach Mannschaften sortiert'!D13</f>
         <v>46172</v>
@@ -4686,8 +4728,11 @@
       <c r="K13" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L13" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B14" s="105">
         <f>'Nach Mannschaften sortiert'!D14</f>
         <v>46179</v>
@@ -4725,8 +4770,11 @@
       <c r="K14" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L14" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B15" s="105">
         <f>'Nach Mannschaften sortiert'!D15</f>
         <v>46096</v>
@@ -4763,8 +4811,11 @@
       <c r="K15" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L15" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B16" s="105">
         <f>'Nach Mannschaften sortiert'!D16</f>
         <v>46102</v>
@@ -4801,8 +4852,11 @@
       <c r="K16" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L16" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="105">
         <f>'Nach Mannschaften sortiert'!D17</f>
         <v>46109</v>
@@ -4839,8 +4893,11 @@
       <c r="K17" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L17" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="105">
         <f>'Nach Mannschaften sortiert'!D18</f>
         <v>46116</v>
@@ -4877,8 +4934,11 @@
       <c r="K18" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L18" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="105">
         <f>'Nach Mannschaften sortiert'!D19</f>
         <v>46124</v>
@@ -4915,8 +4975,11 @@
       <c r="K19" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L19" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="105">
         <f>'Nach Mannschaften sortiert'!D20</f>
         <v>46130</v>
@@ -4953,8 +5016,11 @@
       <c r="K20" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L20" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="105">
         <f>'Nach Mannschaften sortiert'!D21</f>
         <v>46136</v>
@@ -4991,8 +5057,11 @@
       <c r="K21" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L21" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="105">
         <f>'Nach Mannschaften sortiert'!D22</f>
         <v>46144</v>
@@ -5029,8 +5098,11 @@
       <c r="K22" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L22" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="105">
         <f>'Nach Mannschaften sortiert'!D23</f>
         <v>46151</v>
@@ -5067,8 +5139,11 @@
       <c r="K23" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L23" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="105">
         <f>'Nach Mannschaften sortiert'!D24</f>
         <v>46157</v>
@@ -5105,8 +5180,11 @@
       <c r="K24" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L24" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="105">
         <f>'Nach Mannschaften sortiert'!D25</f>
         <v>46166</v>
@@ -5143,8 +5221,11 @@
       <c r="K25" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L25" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="105">
         <f>'Nach Mannschaften sortiert'!D26</f>
         <v>46172</v>
@@ -5181,8 +5262,11 @@
       <c r="K26" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L26" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="105">
         <f>'Nach Mannschaften sortiert'!D27</f>
         <v>46179</v>
@@ -5219,8 +5303,11 @@
       <c r="K27" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L27" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="105">
         <v>46106</v>
       </c>
@@ -5256,8 +5343,11 @@
       <c r="K28" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L28" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="105">
         <f>'Nach Mannschaften sortiert'!D29</f>
         <v>46124</v>
@@ -5295,8 +5385,11 @@
       <c r="K29" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L29" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="105">
         <f>'Nach Mannschaften sortiert'!D30</f>
         <v>46131</v>
@@ -5334,8 +5427,11 @@
       <c r="K30" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L30" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="105">
         <f>'Nach Mannschaften sortiert'!D31</f>
         <v>46138</v>
@@ -5373,8 +5469,11 @@
       <c r="K31" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L31" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="105">
         <f>'Nach Mannschaften sortiert'!D32</f>
         <v>46143</v>
@@ -5412,8 +5511,11 @@
       <c r="K32" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L32" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="105">
         <f>'Nach Mannschaften sortiert'!D33</f>
         <v>46151</v>
@@ -5451,8 +5553,11 @@
       <c r="K33" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L33" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="105">
         <f>'Nach Mannschaften sortiert'!D34</f>
         <v>46159</v>
@@ -5490,8 +5595,11 @@
       <c r="K34" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L34" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="105">
         <f>'Nach Mannschaften sortiert'!D35</f>
         <v>46102</v>
@@ -5529,8 +5637,11 @@
       <c r="K35" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L35" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="105">
         <f>'Nach Mannschaften sortiert'!D36</f>
         <v>46173</v>
@@ -5568,8 +5679,11 @@
       <c r="K36" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L36" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="105">
         <f>'Nach Mannschaften sortiert'!D37</f>
         <v>46180</v>
@@ -5607,8 +5721,11 @@
       <c r="K37" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L37" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="105">
         <f>'Nach Mannschaften sortiert'!D38</f>
         <v>46124</v>
@@ -5646,8 +5763,11 @@
       <c r="K38" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L38" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="105">
         <f>'Nach Mannschaften sortiert'!D39</f>
         <v>46128</v>
@@ -5685,8 +5805,11 @@
       <c r="K39" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L39" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="105">
         <f>'Nach Mannschaften sortiert'!D40</f>
         <v>46137</v>
@@ -5724,8 +5847,11 @@
       <c r="K40" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L40" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="105">
         <f>'Nach Mannschaften sortiert'!D41</f>
         <v>46145</v>
@@ -5763,8 +5889,11 @@
       <c r="K41" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L41" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="105">
         <f>'Nach Mannschaften sortiert'!D42</f>
         <v>46157</v>
@@ -5802,8 +5931,11 @@
       <c r="K42" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L42" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="105">
         <f>'Nach Mannschaften sortiert'!D43</f>
         <v>46165</v>
@@ -5841,8 +5973,11 @@
       <c r="K43" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L43" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="105">
         <f>'Nach Mannschaften sortiert'!D44</f>
         <v>46173</v>
@@ -5880,8 +6015,11 @@
       <c r="K44" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L44" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="105">
         <f>'Nach Mannschaften sortiert'!D45</f>
         <v>46179</v>
@@ -5919,8 +6057,11 @@
       <c r="K45" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L45" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="105">
         <f>'Nach Mannschaften sortiert'!D46</f>
         <v>46145</v>
@@ -5958,8 +6099,11 @@
       <c r="K46" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L46" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="47" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B47" s="105">
         <f>'Nach Mannschaften sortiert'!D47</f>
         <v>46122</v>
@@ -5997,8 +6141,11 @@
       <c r="K47" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L47" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="105">
         <f>'Nach Mannschaften sortiert'!D48</f>
         <v>46131</v>
@@ -6036,8 +6183,11 @@
       <c r="K48" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L48" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B49" s="105">
         <f>'Nach Mannschaften sortiert'!D49</f>
         <v>46137</v>
@@ -6075,8 +6225,11 @@
       <c r="K49" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="50" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L49" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="50" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B50" s="105">
         <v>46151</v>
       </c>
@@ -6113,8 +6266,11 @@
       <c r="K50" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="51" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L50" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B51" s="105">
         <f>'Nach Mannschaften sortiert'!D51</f>
         <v>46173</v>
@@ -6152,8 +6308,11 @@
       <c r="K51" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="52" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L51" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B52" s="105">
         <f>'Nach Mannschaften sortiert'!D52</f>
         <v>46163</v>
@@ -6191,8 +6350,11 @@
       <c r="K52" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="53" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L52" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B53" s="105">
         <f>'Nach Mannschaften sortiert'!D53</f>
         <v>46171</v>
@@ -6230,8 +6392,11 @@
       <c r="K53" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="54" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L53" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B54" s="105">
         <f>'Nach Mannschaften sortiert'!D54</f>
         <v>46188</v>
@@ -6269,8 +6434,11 @@
       <c r="K54" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="55" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L54" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B55" s="105">
         <f>'Nach Mannschaften sortiert'!D55</f>
         <v>46130</v>
@@ -6308,8 +6476,11 @@
       <c r="K55" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="56" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L55" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B56" s="105">
         <f>'Nach Mannschaften sortiert'!D56</f>
         <v>46138</v>
@@ -6347,8 +6518,11 @@
       <c r="K56" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="57" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L56" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B57" s="105">
         <f>'Nach Mannschaften sortiert'!D57</f>
         <v>46145</v>
@@ -6386,8 +6560,11 @@
       <c r="K57" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="58" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L57" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="58" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B58" s="105">
         <f>'Nach Mannschaften sortiert'!D58</f>
         <v>46151</v>
@@ -6425,8 +6602,11 @@
       <c r="K58" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="59" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L58" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B59" s="105">
         <f>'Nach Mannschaften sortiert'!D59</f>
         <v>46167</v>
@@ -6464,8 +6644,11 @@
       <c r="K59" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="60" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L59" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="60" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B60" s="105">
         <f>'Nach Mannschaften sortiert'!D60</f>
         <v>46173</v>
@@ -6503,8 +6686,11 @@
       <c r="K60" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="61" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L60" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="61" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B61" s="105">
         <f>'Nach Mannschaften sortiert'!D61</f>
         <v>46180</v>
@@ -6542,8 +6728,11 @@
       <c r="K61" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="62" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L61" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="62" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B62" s="105">
         <v>46127</v>
       </c>
@@ -6580,8 +6769,11 @@
       <c r="K62" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="63" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L62" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="63" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B63" s="105">
         <f>'Nach Mannschaften sortiert'!D63</f>
         <v>46123</v>
@@ -6619,8 +6811,11 @@
       <c r="K63" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="64" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L63" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="64" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B64" s="105">
         <f>'Nach Mannschaften sortiert'!D64</f>
         <v>46131</v>
@@ -6658,8 +6853,11 @@
       <c r="K64" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="65" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L64" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="65" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B65" s="105">
         <f>'Nach Mannschaften sortiert'!D65</f>
         <v>46135</v>
@@ -6697,8 +6895,11 @@
       <c r="K65" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="66" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L65" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="66" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B66" s="105">
         <v>46155</v>
       </c>
@@ -6734,8 +6935,11 @@
       <c r="K66" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="67" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L66" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="67" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B67" s="105">
         <f>'Nach Mannschaften sortiert'!D67</f>
         <v>46169</v>
@@ -6773,8 +6977,11 @@
       <c r="K67" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="68" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L67" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="68" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B68" s="105">
         <f>'Nach Mannschaften sortiert'!D68</f>
         <v>46164</v>
@@ -6812,8 +7019,11 @@
       <c r="K68" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="69" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L68" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="69" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B69" s="105">
         <f>'Nach Mannschaften sortiert'!D69</f>
         <v>46171</v>
@@ -6851,8 +7061,11 @@
       <c r="K69" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="70" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L69" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="70" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B70" s="105">
         <f>'Nach Mannschaften sortiert'!D70</f>
         <v>46123</v>
@@ -6887,8 +7100,11 @@
       <c r="K70" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="71" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L70" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="71" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B71" s="105">
         <f>'Nach Mannschaften sortiert'!D71</f>
         <v>46130</v>
@@ -6923,8 +7139,11 @@
       <c r="K71" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="72" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L71" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="72" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B72" s="105">
         <f>'Nach Mannschaften sortiert'!D72</f>
         <v>46137</v>
@@ -6959,8 +7178,11 @@
       <c r="K72" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="73" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L72" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="73" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B73" s="105">
         <f>'Nach Mannschaften sortiert'!D73</f>
         <v>46151</v>
@@ -6995,8 +7217,11 @@
       <c r="K73" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="74" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L73" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="74" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B74" s="105">
         <f>'Nach Mannschaften sortiert'!D74</f>
         <v>46194</v>
@@ -7031,8 +7256,11 @@
       <c r="K74" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="75" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L74" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="75" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B75" s="105">
         <f>'Nach Mannschaften sortiert'!D75</f>
         <v>46123</v>
@@ -7067,8 +7295,11 @@
       <c r="K75" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="76" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L75" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="76" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B76" s="105">
         <f>'Nach Mannschaften sortiert'!D76</f>
         <v>46137</v>
@@ -7103,8 +7334,11 @@
       <c r="K76" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="77" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L76" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="77" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B77" s="105">
         <f>'Nach Mannschaften sortiert'!D77</f>
         <v>46144</v>
@@ -7139,8 +7373,11 @@
       <c r="K77" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="78" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L77" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="78" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B78" s="105">
         <f>'Nach Mannschaften sortiert'!D78</f>
         <v>46151</v>
@@ -7175,8 +7412,11 @@
       <c r="K78" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="79" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L78" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="79" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B79" s="105">
         <f>'Nach Mannschaften sortiert'!D79</f>
         <v>46180</v>
@@ -7211,8 +7451,11 @@
       <c r="K79" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="80" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L79" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="80" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B80" s="105">
         <f>'Nach Mannschaften sortiert'!D80</f>
         <v>46123</v>
@@ -7247,8 +7490,11 @@
       <c r="K80" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="81" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L80" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="81" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B81" s="105">
         <f>'Nach Mannschaften sortiert'!D81</f>
         <v>46131</v>
@@ -7283,8 +7529,11 @@
       <c r="K81" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="82" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L81" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="82" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B82" s="105">
         <f>'Nach Mannschaften sortiert'!D82</f>
         <v>46143</v>
@@ -7319,8 +7568,11 @@
       <c r="K82" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="83" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L82" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="83" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B83" s="105">
         <f>'Nach Mannschaften sortiert'!D83</f>
         <v>46151</v>
@@ -7355,8 +7607,11 @@
       <c r="K83" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="84" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L83" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="84" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B84" s="105">
         <f>'Nach Mannschaften sortiert'!D84</f>
         <v>46187</v>
@@ -7391,8 +7646,11 @@
       <c r="K84" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="85" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L84" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="85" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B85" s="105">
         <f>'Nach Mannschaften sortiert'!D85</f>
         <v>46111</v>
@@ -7426,8 +7684,11 @@
       <c r="K85" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="86" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L85" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="86" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B86" s="105">
         <f>'Nach Mannschaften sortiert'!D86</f>
         <v>46112</v>
@@ -7461,8 +7722,11 @@
       <c r="K86" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="87" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L86" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="87" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B87" s="105">
         <f>'Nach Mannschaften sortiert'!D87</f>
         <v>46113</v>
@@ -7496,8 +7760,11 @@
       <c r="K87" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="88" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L87" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="88" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B88" s="105">
         <f>'Nach Mannschaften sortiert'!D88</f>
         <v>46186</v>
@@ -7529,8 +7796,11 @@
       <c r="K88" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="89" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L88" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="89" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B89" s="105">
         <f>'Nach Mannschaften sortiert'!D89</f>
         <v>46256</v>
@@ -7567,8 +7837,11 @@
       <c r="K89" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="90" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L89" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="90" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B90" s="105">
         <v>46124</v>
       </c>
@@ -7600,8 +7873,11 @@
       <c r="K90" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="91" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L90" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="91" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B91" s="105">
         <v>46119</v>
       </c>
@@ -7631,6 +7907,9 @@
       </c>
       <c r="K91" t="s">
         <v>158</v>
+      </c>
+      <c r="L91" t="s">
+        <v>245</v>
       </c>
     </row>
   </sheetData>

</xml_diff>